<commit_message>
Update EDB prices for July 23
</commit_message>
<xml_diff>
--- a/edb_data/Nand Flash.xlsx
+++ b/edb_data/Nand Flash.xlsx
@@ -696,19 +696,13 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -33248,13 +33242,13 @@
       </c>
     </row>
     <row r="2908" spans="1:3">
-      <c r="A2908" s="5">
+      <c r="A2908" s="3">
         <v>41429</v>
       </c>
-      <c r="B2908" s="6">
+      <c r="B2908" s="4">
         <v>6.158</v>
       </c>
-      <c r="C2908" s="6">
+      <c r="C2908" s="4">
         <v>3.946</v>
       </c>
     </row>

</xml_diff>